<commit_message>
fix lỗi imis sang MSC
</commit_message>
<xml_diff>
--- a/data/Bang_Tham_Dinh_Du_Toan.xlsx
+++ b/data/Bang_Tham_Dinh_Du_Toan.xlsx
@@ -500,7 +500,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Bang_Tham_Dinh_Du_Toan (3) - Bản Mới</t>
+          <t>Bang_Tham_Dinh_Du_Toan (3) - Bản Mới - Bản Mới</t>
         </is>
       </c>
     </row>
@@ -635,18 +635,13 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>TỔ THẨM ĐỊNH NHÀ MÁY NHIỆT ĐIỆN VĨNH TÂN 4
-TỔ THẨM ĐỊNH DỰ TOÁN
-BÁO CÁO THUYẾT MINH THẨM ĐỊNH ĐƠN GIÁ VẬT TƯ
-Đơn vị yêu cầu: NMNĐ Vĩnh Tân 4
-Mã ERP: 3.82.63.134.ENG.00.000 | Số lượng: 4 Cái
-Tên vật tư: Module đầu vào input IUX 760 MI – Điện áp hoạt động: 17-28VDC
-Partno: 908531 | Hãng sản xuất: Minimax
-Đơn giá trình thẩm định: 13.559.000 đ/Cái
-1. TỔNG HỢP ĐÁNH GIÁ THẨM ĐỊNH MỤC
-Tổ Thẩm định tiến hành đối chiếu đơn giá trình thẩm định đối với mặt hàng Module đầu vào input IUX 760 MI (Partno: 908531, hãng Minimax) trên 5 cơ sở chứng cứ thu thập được, cụ thể:
-(1) Báo giá gốc thương mại; (2) Lịch sử mua sắm trên ERP Vĩnh Tân 4; (3) Cơ sở dữ liệu mua sắm EVN IMIS của các Đơn vị Phát điện trong Tập đoàn; (4) Cơ sở dữ liệu Mua sắm Công (e-GP); (5) Khảo sát giá thương mại điện tử trên các sàn giao dịch và Internet.
-Kết quả tổng hợp cho thấy đơn giá trình 13.559.000 đ/Cái là mức chào thấp nhất từ nhà thầu trong báo giá thương mại hiện tại; tuy nhiên khi đối chiếu với lị</t>
+          <t>TỔNG HỢP 5 CƠ SỞ CHỨNG CỨ (Đã rà soát nhanh):
+• Cơ sở 1 (Báo Giá Gốc): Báo giá chào thấp nhất: 13.559.000 đ/Cái (DTL 19.8.2026. xlsx)
+• Cơ sở 2 (ERP Vĩnh Tân 4): Lịch sử nhập kho ERP Vĩnh Tân 4: 6.015.000 đ/Cái (HĐ: Nhập kho vật tư (HĐ: 115/2023. Ttr 2562/KHVT) theo hóa đơn số 00000041. 42. 43. 44. 45. 46 ngày 30.08.2024 ngày 2024-10-31. SL: 117 Cái); Các đợt nhập khác: 17.670.000 đ
+• Cơ sở 3 (EVN IMIS): Trong khoảng thời gian tra cứu từ ngày 01/01/2023 đến nay, qua đối chiếu CSDL EVN IMIS theo từ khóa [908531], vật tư chưa tìm thấy dữ liệu mua sắm tương đương trên CSDL EVN IMIS.
+• Cơ sở 4 (Mua Sắm Công e-GP): Đã tra cứu từ khóa [Module đầu vào input IUX 760 MI] trên Mạng Đấu thầu Quốc gia nhưng chưa ghi nhận kết quả trúng thầu tương tự.
+• Cơ sở 5 (TMĐT &amp; Tham Khảo Web): Vật tư đặc thù - Yêu cầu báo giá riêng (Contact for Quote)
+KẾT LUẬN: Đơn giá tham chiếu mốc thấp nhất đề xuất là 6.015.000 đ/Cái.</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr"/>
@@ -710,8 +705,13 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Ý KIẾN ĐÁNH GIÁ &amp; BẢN THUYẾT MINH THẨM ĐỊNH CỦA TỔ THẨM ĐỊNH DỰ TOÁN
-Căn cứ tính chất kỹ thuật, thương hiệu sản xuất và chứng cứ thu thập tại 05 cơ sở thẩm định, Tổ Thẩm định dự toán – Nhà máy Nhiệt điện Vĩnh Tân 4 thống nhất nội dung đánh giá đối với vật tư: Nút nhấn khẩn cấp Discovery Manual Call Point, Part no: 58100-953, nguồn cấp 17 – 28VDC, cấp bảo vệ IP67, nhà sản xuất Apollo (Mã ERP: 3.34.40.024.ENG.00.000), số lượng 01 cái, đơn giá trình thẩm định 14.208.000 đ</t>
+          <t>TỔNG HỢP 5 CƠ SỞ CHỨNG CỨ (Đã rà soát nhanh):
+• Cơ sở 1 (Báo Giá Gốc): Báo giá chào thấp nhất: 14.208.000 đ/Cái (CÔNG TY CỔ PHẦN XÂY DỰNG VÀ KỸ THUẬT THĂNG LONG)
+• Cơ sở 2 (ERP Vĩnh Tân 4): Lịch sử nhập kho ERP Vĩnh Tân 4: 7.000.000 đ/Cái (HĐ: Nhập kho vật tư (QĐ:161) theo hóa đơn số 0000221 ngày 26.03.2021 ngày 2021-04-14. SL: 1 Cái)
+• Cơ sở 3 (EVN IMIS): Trong khoảng thời gian tra cứu từ ngày 01/01/2023 đến nay, qua đối chiếu CSDL EVN IMIS theo từ khóa [58100-953], vật tư chưa tìm thấy dữ liệu mua sắm tương đương trên CSDL EVN IMIS.
+• Cơ sở 4 (Mua Sắm Công e-GP): Đã tra cứu từ khóa [Nút nhấn khẩn cấp - Discovery manual call point, Part no: 58100-953] trên Mạng Đấu thầu Quốc gia nhưng chưa ghi nhận kết quả trúng thầu tương tự.
+• Cơ sở 5 (TMĐT &amp; Tham Khảo Web): Vật tư đặc thù - Yêu cầu báo giá riêng (Contact for Quote)
+KẾT LUẬN: Đơn giá tham chiếu mốc thấp nhất đề xuất là 7.000.000 đ/Cái.</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr"/>
@@ -863,7 +863,7 @@
         <is>
           <t># THUYẾT MINH THẨM ĐỊNH MỤC STT 4
 ## TỔNG HỢP ĐÁNH GIÁ THẨM ĐỊNH MỤC
-Tổ Thẩm định thực hiện thẩm định đánh giá sau cùng đối với vật tư Solenoid van 600250-70900533 (Hãng SX: Bray International, số lượng 5 Bộ). Đơn giá dự toán trình là 64.000.000 đ/Bộ, cao hơn +610.4% so với đơn giá tham chiếu thấp nhất hợp lệ (9.009.300 đ từ Cơ sở 5). Tổ Thẩm định đề xuất điều chỉnh đơn giá theo giá thị trường quốc tế đã tính đủ chi phí nhập cảnh &amp; vận chuyển DDP Vĩ</t>
+Tổ Thẩm định thự</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr"/>
@@ -933,7 +933,7 @@
 • Đánh giá Mức độ Hợp lý Đơn giá: 100/100 điểm (🟢 Rất Hợp Lý (Đơn giá trình &lt;= Giá thấp nhất công khai)).
 CƠ SỞ THẨM ĐỊNH THỐNG NHẤT 5 CƠ SỞ CHỨNG CỨ:
 - Cơ sở 1 (Báo Giá Gốc): Đã đối chiếu các báo giá thương mại cạnh tranh trong Hồ sơ trình; ghi nhận đơn giá chào thấp nhất là 1.500.000 VNĐ/Cái từ CÔNG TY CỔ PHẦN XÂY DỰNG VÀ KỸ THUẬT THĂNG LONG (Trang 1 Báo giá); đơn giá chào đối chiếu khớp 100% với đơn giá dự toán trình.
-- Cơ sở 2 (ERP Vĩnh Tân 4): Qua rà soát CSDL Kế toán ERP của NMNĐ Vĩnh Tân 4 theo từ khóa [Spiral Wound Gasket DN200 PN40], các kết quả tra cứu không có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Thẩm định viên không áp dụng CSDL ERP làm căn cứ so sánh đơn giá cho mục này.
+- Cơ sở 2 (ERP Vĩnh Tân 4): Qua rà soát CSDL lịch sử mua sắm ERP của NMNĐ Vĩnh Tân 4 theo từ khóa [Spiral Wound Gasket DN200 PN40], các kết quả tra cứu không có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Thẩm định viên không áp dụng CSDL ERP làm căn cứ so sánh đơn giá cho mục này.
 - Cơ sở 3 (EVN IMIS): Tra cứu theo từ khóa [Spiral Wound Gasket DN200 PN40] trên CSDL Hợp đồng mua sắm toàn ngành EVN IMIS (2023-2026); kết quả đã đối soát toàn CSDL EVN: 0 bản ghi phù hợp (không phát sinh mua sắm tương đương).
 - Cơ sở 4 (Mua Sắm Công e-GP): Tra cứu theo từ khóa [Spiral Wound Gasket] trên Cổng Mạng Đấu thầu Quốc gia (muasamcong.mpi.gov.vn); kết quả đã rà soát e-GP: vật tư đặc thù, không ghi nhận gói thầu mua sắm tương đồng.
 - Cơ sở 5 (Thương Mại Điện Tử): Tra cứu theo từ khóa [Spiral Wound Gasket DN200 PN40] trên các cổng Internet &amp; Sàn TMĐT (eBay, Misumi, Google Web); kết quả ghi nhận vật tư thuộc danh mục thiết bị đặc thù công nghiệp, các trang web/nhà cung cấp không niêm yết đơn giá thương mại công khai (yêu cầu gửi thư yêu cầu báo giá riêng - Contact for Quote).
@@ -1236,9 +1236,11 @@
 • Đánh giá Mức độ Hợp lý Đơn giá: 100/100 điểm (🟢 Rất Hợp Lý (Đơn giá trình &lt;= Giá thấp nhất công khai)).
 CƠ SỞ THẨM ĐỊNH THỐNG NHẤT 5 CƠ SỞ CHỨNG CỨ:
 - Cơ sở 1 (Báo Giá Gốc): Đã đối chiếu các báo giá thương mại cạnh tranh trong Hồ sơ trình; ghi nhận đơn giá chào thấp nhất là 1.315.000 VNĐ/Cái từ CÔNG TY CỔ PHẦN XÂY DỰNG VÀ KỸ THUẬT THĂNG LONG (Trang 2 Báo giá); đơn giá chào đối chiếu khớp 100% với đơn giá dự toán trình.
-- Cơ sở 2 (ERP Vĩnh Tân 4): Qua rà soát CSDL Kế toán ERP của NMNĐ Vĩnh Tân 4 theo từ khóa [Elbow union], các kết quả tra cứu không có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Thẩm định viên không áp dụng CSDL ERP làm căn cứ so sánh đơn giá cho mục này.
+- Cơ sở 2 (ERP Vĩnh Tân 4): Qua rà soát CSDL lịch sử mua sắm ERP của NMNĐ Vĩnh Tân 4 theo từ khóa [Elbow union], các kết quả tra cứu không có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Thẩm định viên không áp dụng CSDL ERP làm căn cứ so sánh đơn giá cho mục này.
 - Cơ sở 3 (EVN IMIS): Tra cứu theo từ khóa [10-PL A3C] trên CSDL Hợp đồng mua sắm toàn ngành EVN IMIS (2023-2026); kết quả đã đối soát toàn CSDL EVN: 0 bản ghi phù hợp (không phát sinh mua sắm tương đương).
-- Cơ sở 4 (Mua Sắm Công e-GP): Tra cứu theo từ khóa [W 10-PL A3C] trên Cổng Mạng Đấu thầu Quố</t>
+- Cơ sở 4 (Mua Sắm Công e-GP): Tra cứu theo từ khóa [W 10-PL A3C] trên Cổng Mạng Đấu thầu Quốc gia (muasamcong.mpi.gov.vn); kết quả đã rà soát e-GP: vật tư đặc thù, không ghi nhận gói thầu mua sắm tương đồng.
+- Cơ sở 5 (Thương Mại Điện Tử): Tra cứu theo từ khóa [10-PL A3C] trên các cổng Internet &amp; Sàn TMĐT (eBay, Misumi, Google Web); kết quả ghi nhận vật tư thuộc danh mục thiết bị đặc thù công nghiệp, các trang web/nhà cung cấp không niêm yết đơn giá thương mại công khai (yêu cầu gửi thư yêu cầu báo giá riêng - Contact for Quote).
+KẾT LUẬN THẨM ĐỊNH: Đơn giá trình phù hợp với mặt bằng giá thị trường. Đề xuất phê duyệt giữ nguyên đơn giá trình là 1.315.000 VNĐ/Cái.</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr"/>
@@ -1329,7 +1331,7 @@
 Đơn giá trình thẩm định 1.508.000 đ/Cái cao hơn **+80,2%** so với đơn giá tham chiếu thấp nhất hợp lệ là 836.800 đ/Cái (mức chênh tuyệt đối 671.200 đ/Cái). Với đặc tính kỹ thuật của cụm vật tư chuyên dụng G7, biên độ chênh lệch này vượt khá xa ngưỡng biến động hợp lý thường gặp (thông thường dưới 15–20%) giữa các báo giá cùng chủng loại, cùng xuất xứ. Tổ Thẩm định nhận thấy mức giá trình chưa có cơ sở thuyết phục để chứng minh tính hợp lý và cần được đàm phán điều chỉnh về mặt bằng giá thị trường.
 **3. Đối chiếu 05 cơ sở chứng cứ thẩm định**
 - **Cơ sở 1 – Báo giá gốc (thương mại):** Tổ Thẩm định đã đối chiếu các báo giá thương mại thu thập được; mức chào thấp nhất hợp lệ là **836.800 đ/Cái** từ Nhà thầu chào giá cạnh tranh. Đơn giá trình 1.508.000 đ/Cái không phải mức thấp nhất trên thị trường, chênh lệch +80,2% cho thấy dấu hiệu bất thường cần đàm phán.
-- **Cơ sở 2 – Cơ sở dữ liệu ERP Nhà máy Nhiệt điện Vĩnh Tân 4:** Qua rà soát CSDL Kế toán ERP, không có kết quả tra cứu nào có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Tổ Thẩm định **không áp dụng** CSDL ERP làm căn cứ so sánh đơn giá cho mục này.
+- **Cơ sở 2 – Cơ sở dữ liệu ERP Nhà máy Nhiệt điện Vĩnh Tân 4:** Qua rà soát CSDL lịch sử mua sắm ERP, không có kết quả tra cứu nào có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Tổ Thẩm định **không áp dụng** CSDL ERP làm căn cứ so sánh đơn giá cho mục này.
 - **Cơ sở 3 – Cơ sở dữ liệu EVN IMIS:** Tra cứu theo từ khóa **[DPR 10-L/S]** cho thấy các kết quả tìm thấy không tương đồng về quy cách/chủng loại với vật tư dự toán. Tổ Thẩm định **không áp dụng** làm căn cứ thẩm định.
 - **Cơ sở 4 – Hệ thống Mua sắm Công (e-GP) – muasamcong.mpi.gov.vn:** Tra cứu từ khóa **[126091]** tại thời điểm 18:31 ngày 07/09/2026 **chưa ghi nhận** kết quả trúng thầu tương tự. Tổ Thẩm định ghi nhận sự hạn chế dữ liệu tham chiếu từ kênh này.
 - **Cơ sở 5 – Thương mại điện tử:** Dữ liệu không khả dụng/không có kết quả phù hợp để đối chiếu; Tổ Thẩm định **không áp dụng** làm căn cứ so sánh đơn giá.
@@ -1407,13 +1409,23 @@
       <c r="I15" s="7" t="n">
         <v>24100000</v>
       </c>
-      <c r="J15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>TỔNG HỢP 5 CƠ SỞ CHỨNG CỨ (Đã rà soát nhanh):
+• Cơ sở 1 (Báo Giá Gốc): Chưa nạp dữ liệu Báo giá gốc
+• Cơ sở 2 (ERP Vĩnh Tân 4): Lịch sử nhập kho ERP Vĩnh Tân 4: 64.001.100 đ/Mét (HĐ: Nhập kho vật tư (HĐ: 40/2025) theo hóa đơn số 1956 ngày 30.10.2025 ngày 2025-12-12. SL: 3 Mét); Các đợt nhập khác: 16.649.700 đ, 11.181.019 đ
+• Cơ sở 3 (EVN IMIS): Trong khoảng thời gian tra cứu từ ngày 01/01/2023 đến nay, qua đối chiếu CSDL EVN IMIS theo từ khóa [B-210-2394], vật tư chưa tìm thấy dữ liệu mua sắm tương đương trên CSDL EVN IMIS.
+• Cơ sở 4 (Mua Sắm Công e-GP): Đã tra cứu từ khóa [Ống B-210-2394/1] trên Mạng Đấu thầu Quốc gia nhưng chưa ghi nhận kết quả trúng thầu tương tự.
+• Cơ sở 5 (TMĐT &amp; Tham Khảo Web): Vật tư đặc thù - Yêu cầu báo giá riêng (Contact for Quote)
+KẾT LUẬN: Đơn giá tham chiếu mốc thấp nhất đề xuất là 64.001.100 đ/Mét.</t>
+        </is>
+      </c>
       <c r="K15" s="6" t="inlineStr"/>
       <c r="L15" s="7" t="n">
-        <v>1205000</v>
+        <v>64001100</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>24100000</v>
+        <v>1280022000</v>
       </c>
       <c r="N15" s="7" t="n">
         <v>0</v>
@@ -1479,18 +1491,32 @@
       <c r="I16" s="7" t="n">
         <v>117600000</v>
       </c>
-      <c r="J16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>TỔNG HỢP 5 CƠ SỞ CHỨNG CỨ (Đã rà soát nhanh):
+• Cơ sở 1 (Báo Giá Gốc): Báo giá chào thấp nhất: 117.600.000 đ/Cái (CÔNG TY CỔ PHẦN XÂY DỰNG VÀ KỸ THUẬT THĂNG LONG)
+• Cơ sở 2 (ERP Vĩnh Tân 4): Lịch sử nhập kho ERP Vĩnh Tân 4: 57.465.833 đ/Cái (HĐ: Nhập kho vật tư (HĐ: 65/2024) theo hóa đơn số 00000008 ngày 05.06.2025 ngày 2025-07-03. SL: 2 Cái); Các đợt nhập khác: 169.000.000 đ
+• Cơ sở 3 (EVN IMIS): Trong khoảng thời gian tra cứu từ ngày 01/01/2023 đến nay, qua đối chiếu CSDL EVN IMIS theo từ khóa [RTNC3], vật tư chưa tìm thấy dữ liệu mua sắm tương đương trên CSDL EVN IMIS.
+• Cơ sở 4 (Mua Sắm Công e-GP): Đã tra cứu từ khóa [Cảm biến đo khối lượng (Loadcell), model: RTNC3/10T] trên Mạng Đấu thầu Quốc gia nhưng chưa ghi nhận kết quả trúng thầu tương tự.
+• Cơ sở 5 (TMĐT &amp; Tham Khảo Web): Vật tư đặc thù - Yêu cầu báo giá riêng (Contact for Quote)
+KẾ</t>
+        </is>
+      </c>
       <c r="K16" s="6" t="inlineStr"/>
       <c r="L16" s="7" t="n">
-        <v>117600000</v>
+        <v>113232916.5</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>117600000</v>
+        <v>113232916</v>
       </c>
       <c r="N16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="6" t="inlineStr"/>
+        <v>4367084</v>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
           <t>3.96.13.021.GER.00.000 | Thay thế 01 cảm biến đo khối lượng (Loadcell) bồn chứa khí CO2 – Tổ máy S3 bị hư hỏng | BBKT 510/2026/VH-VT4. Vật tư không có trong KH SXKD 2026.</t>
@@ -1910,7 +1936,21 @@
       <c r="I23" s="7" t="n">
         <v>675500000</v>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>TỔNG HỢP ĐÁNH GIÁ THẨM ĐỊNH MỤC: Ống khí nén/ tube, Model: SS-T6-S-065-20, OD: 3/8 inch, Length: 6m (Mã ERP: 2.46.35.037.CHN.00.000).
+• Đơn giá trình thẩm định: 19.300.000 VNĐ (Số lượng: 35 Cái).
+• Đánh giá Chứng cứ Thẩm định: Đạt 60/100 điểm (Hạng B - 3/5 cơ sở chứng cứ đã nạp).
+• Đánh giá Mức độ Hợp lý Đơn giá: 85/100 điểm (🟡 Hợp Lý (Nằm trong biên độ giá trung bình thị trường)).
+CƠ SỞ THẨM ĐỊNH THỐNG NHẤT 5 CƠ SỞ CHỨNG CỨ:
+- Cơ sở 1 (Báo Giá Gốc): Đã đối chiếu các báo giá thương mại cạnh tranh trong Hồ sơ trình; ghi nhận đơn giá chào thấp nhất là 18.522.000 VNĐ/Cái từ CÔNG TY TNHH THƯƠNG MẠI KỸ THUẬT NĂNG LƯỢNG AN HIẾU (Trang 3 Báo giá); đơn giá chào đối chiếu thấp hơn 778.000 VNĐ/Cái so với đơn giá trình.
+- Cơ sở 2 (ERP Vĩnh Tân 4): Tra cứu theo từ khóa [2.46.35.037.CHN.00.000] trong CSDL lịch sử mua sắm ERP nội bộ nhà máy Vĩnh Tân 4; ghi nhận đơn giá nhập kho gần nhất là 21.200.000 VNĐ/Cái theo HĐ Nhập kho vật tư (HĐ: 120/2024) theo hóa đơn số 00000008 ngày 13.01.2025 (ký ngày 2025-01-16 00:00:00, cách đây 20 tháng ~ 1.7 năm - quá 12 tháng, tốc độ tăng giá bình quân -5.4%/năm so với CPI ~5.0%/năm).
+- Cơ sở 3 (EVN IMIS): Chưa đối chiếu CSDL Hợp đồng mua sắm toàn ngành EVN IMIS.
+- Cơ sở 4 (Mua Sắm Công e-GP): Tra cứu theo từ khóa [SS-T6-S-065-20] trên Cổng Mạng Đấu thầu Quốc gia (muasamcong.mpi.gov.vn); ghi nhận đơn giá trúng thầu công khai tham chiếu là 27.390.000 VNĐ/Cái (Nhà thầu Swagelok).
+- Cơ sở 5 (Thương Mại Điện Tử): Tra cứu theo từ khóa [Ống khí nén/ tube, Model: SS-T6-S-065-20, OD: 3/8 inch, Length: 6m] trên các cổng Internet &amp; Sàn TMĐT (eBay, Misumi, Google Web); kết quả ghi nhận vật tư thuộc danh mục thiết bị đặc thù công nghiệp, các trang web/nhà cung cấp không niêm yết đơn giá thương mại công khai (yêu cầu gửi thư yêu cầu báo giá riêng - Contact for Quote).
+KẾT LUẬN THẨM ĐỊNH: Đề xuất duyệt đơn giá thẩm định thống nhất là 18.522.000 VNĐ/Cái. Tiết kiệm dự toán 27.230.000 VNĐ (-4.0%).</t>
+        </is>
+      </c>
       <c r="K23" s="6" t="inlineStr"/>
       <c r="L23" s="7" t="n">
         <v>18522000</v>
@@ -1921,7 +1961,11 @@
       <c r="N23" s="7" t="n">
         <v>27230000</v>
       </c>
-      <c r="O23" s="6" t="inlineStr"/>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>Cơ sở 1: Báo giá nộp kèm</t>
+        </is>
+      </c>
       <c r="P23" s="6" t="inlineStr">
         <is>
           <t>2.46.35.037.CHN.00.000 | Khu vực hoàn nguyên xử lý nước230/2026/PXH-VT4 | Không có trong KHSXKD 2026</t>
@@ -5642,16 +5686,26 @@
       <c r="I86" s="7" t="n">
         <v>5236608000</v>
       </c>
-      <c r="J86" s="6" t="inlineStr"/>
+      <c r="J86" s="6" t="inlineStr">
+        <is>
+          <t>TỔNG HỢP 5 CƠ SỞ CHỨNG CỨ (Đã rà soát nhanh):
+• Cơ sở 1 (Báo Giá Gốc): Báo giá chào thấp nhất: 1.300.000 đ/Bộ (CÔNG TY TNHH THƯƠNG MẠI KỸ THUẬT NĂNG LƯỢNG AN HIẾU)
+• Cơ sở 2 (ERP Vĩnh Tân 4): Lịch sử nhập kho ERP Vĩnh Tân 4: 1.845.000.000 đ/Bộ (HĐ: Nhập kho vật tư (HĐ: 32/2025) theo hóa đơn số 00000181 ngày 26.11.2025 ngày 2025-12-04. SL: 3 Bộ); Các đợt nhập khác: 1.293.213.000 đ
+• Cơ sở 3 (EVN IMIS): Trong khoảng thời gian tra cứu từ ngày 01/01/2023 đến nay, qua đối chiếu CSDL EVN IMIS theo từ khóa [Lining Plate (Compound Armour], vật tư chưa tìm thấy dữ liệu mua sắm tương đương trên CSDL EVN IMIS.
+• Cơ sở 4 (Mua Sắm Công e-GP): Đã tra cứu từ khóa [Lining Plate (Compound Armour Plate) Tấm lót thân máy nghiền than] trên Mạng Đấu thầu Quốc gia nhưng chưa ghi nhận kết quả trúng thầu tương tự.
+• Cơ sở 5 (TMĐT &amp; Tham Khảo Web): Vật tư đặc thù - Yêu cầu báo giá riêng (Contact for Quote)
+KẾT LUẬN: Đơn giá tham chiếu mốc thấp nhất đề xuất là 1.300.000 đ/Bộ.</t>
+        </is>
+      </c>
       <c r="K86" s="6" t="inlineStr"/>
       <c r="L86" s="7" t="n">
-        <v>2618304000</v>
+        <v>1300000</v>
       </c>
       <c r="M86" s="7" t="n">
-        <v>5236608000</v>
+        <v>2600000</v>
       </c>
       <c r="N86" s="7" t="n">
-        <v>0</v>
+        <v>5234008000</v>
       </c>
       <c r="O86" s="6" t="inlineStr"/>
       <c r="P86" s="6" t="inlineStr">
@@ -6571,7 +6625,7 @@
         <is>
           <t>TỔNG HỢP 5 CƠ SỞ CHỨNG CỨ (Đã rà soát nhanh):
 • Cơ sở 1 (Báo Giá Gốc): Báo giá chào thấp nhất: 750.000.000 đ/Cái (08-27-26. BV-VT 4. . 1.620.000.000 vnd. 3 trang. R1.)
-• Cơ sở 2 (ERP Vĩnh Tân 4): Vật tư chưa có lịch sử mua sắm/nhập kho trong CSDL Kế toán ERP của NMNĐ Vĩnh Tân 4.
+• Cơ sở 2 (ERP Vĩnh Tân 4): Vật tư chưa có lịch sử mua sắm/nhập kho trong CSDL lịch sử mua sắm ERP của NMNĐ Vĩnh Tân 4.
 • Cơ sở 3 (EVN IMIS): Trong khoảng thời gian tra cứu từ ngày 01/01/2023 đến nay, qua đối chiếu CSDL EVN IMIS theo từ khóa [TP400 PP], vật tư chưa tìm thấy dữ liệu mua sắm tương đương trên CSDL EVN IMIS.
 • Cơ sở 4 (Mua Sắm Công e-GP): Đã tra cứu từ khóa [Động cơ và bơm NAOH, Type: TP400 PP, FCA 112 MC-2/HE, Công suất: 5,5kW] trên Mạng Đấu thầu Quốc gia nhưng chưa ghi nhận kết quả trúng thầu tương tự.
 • Cơ sở 5 (TMĐT &amp; Tham Khảo Web): Vật tư đặc thù - Yêu cầu báo giá riêng (Contact for Quote)
@@ -6807,26 +6861,34 @@
       </c>
       <c r="J106" s="6" t="inlineStr">
         <is>
-          <t>TỔNG HỢP 5 CƠ SỞ CHỨNG CỨ (Đã rà soát nhanh):
-• Cơ sở 1 (Báo Giá Gốc): Báo giá chào thấp nhất: 750.000.000 đ/Cái (08-27-26. BV-VT 4. . 1.620.000.000 vnd. 3 trang. R1.)
-• Cơ sở 2 (ERP Vĩnh Tân 4): Vật tư chưa có lịch sử mua sắm/nhập kho trong CSDL Kế toán ERP của NMNĐ Vĩnh Tân 4.
-• Cơ sở 3 (EVN IMIS): Trong khoảng thời gian tra cứu từ ngày 01/01/2023 đến nay, qua đối chiếu CSDL EVN IMIS theo từ khóa [TP400 PP], vật tư chưa tìm thấy dữ liệu mua sắm tương đương trên CSDL EVN IMIS.
-• Cơ sở 4 (Mua Sắm Công e-GP): Đã tra cứu từ khóa [Động cơ và bơm NAOH, Type: TP400 PP, FCA 112 MC-2/HE, Công suất: 5,5kW] trên Mạng Đấu thầu Quốc gia nhưng chưa ghi nhận kết quả trúng thầu tương tự.
-• Cơ sở 5 (TMĐT &amp; Tham Khảo Web): Vật tư đặc thù - Yêu cầu báo giá riêng (Contact for Quote)
-KẾT LUẬN: Đơn giá tham chiếu mốc thấp nhất đề xuất là 750.000.000 đ/Bộ.</t>
+          <t>TỔNG HỢP ĐÁNH GIÁ THẨM ĐỊNH MỤC: Phôi inconel 718, đường kính D50mm (Mã ERP: Chưa có mã vật tư).
+• Đơn giá trình thẩm định: 90.000.000 VNĐ (Số lượng: 1 Mét).
+• Đánh giá Chứng cứ Thẩm định: Đạt 100/100 điểm (Hạng A - 5/5 cơ sở chứng cứ đã nạp).
+• Đánh giá Mức độ Hợp lý Đơn giá: 100/100 điểm (🟢 Rất Hợp Lý (Đơn giá trình &lt;= Giá thấp nhất công khai)).
+CƠ SỞ THẨM ĐỊNH THỐNG NHẤT 5 CƠ SỞ CHỨNG CỨ:
+- Cơ sở 1 (Báo Giá Gốc): Đã đối chiếu các báo giá thương mại cạnh tranh trong Hồ sơ trình; ghi nhận đơn giá chào thấp nhất là 90.000.000 VNĐ/Mét từ CÔNG TY TNHH THƯƠNG MẠI KỸ THUẬT NĂNG LƯỢNG AN HIẾU (Trang 2 Báo giá); đơn giá chào đối chiếu khớp 100% với đơn giá dự toán trình.
+- Cơ sở 2 (ERP Vĩnh Tân 4): Qua rà soát CSDL lịch sử mua sắm ERP của NMNĐ Vĩnh Tân 4 theo từ khóa [Phôi inconel 718], các kết quả tra cứu không có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Thẩm định viên không áp dụng CSDL ERP làm căn cứ so sánh đơn giá cho mục này.
+- Cơ sở 3 (EVN IMIS): Tra cứu theo từ khóa [Phôi inconel 718, đường kính D50mm] trên CSDL Hợp đồng mua sắm toàn ngành EVN IMIS (2023-2026); kết quả đã đối soát toàn CSDL EVN: 0 bản ghi phù hợp (không phát sinh mua sắm tương đương).
+- Cơ sở 4 (Mua Sắm Công e-GP): Qua rà soát Cổng Mạng Đấu thầu Quốc gia e-GP (muasamcong.mpi.gov.vn) theo từ khóa [Phôi inconel 718], các kết quả tra cứu không có tính chất kỹ thuật và quy cách tương đồng phù hợp với vật tư đang xét. Thẩm định viên không áp dụng CSDL Mua sắm công làm căn cứ so sánh đơn giá cho mục này.
+- Cơ sở 5 (Thương Mại Điện Tử): Đã tra cứu từ khóa [Phôi inconel 718, đường kính D50mm] trên các cổng Internet &amp; Sàn TMĐT (eBay, Misumi, Google Web); kết quả ghi nhận vật tư thuộc danh mục thiết bị đặc thù công nghiệp, các trang web/nhà cung cấp không niêm yết đơn giá thương mại công khai (yêu cầu gửi thư yêu cầu báo giá riêng - Contact for Quote).
+KẾT LUẬN THẨM ĐỊNH: Đơn giá trình phù hợp với mặt bằng giá thị trường. Đề xuất phê duyệt giữ nguyên đơn giá trình là 90.000.000 VNĐ/Mét.</t>
         </is>
       </c>
       <c r="K106" s="6" t="inlineStr"/>
       <c r="L106" s="7" t="n">
-        <v>750000000</v>
+        <v>90000000</v>
       </c>
       <c r="M106" s="7" t="n">
-        <v>750000000</v>
+        <v>90000000</v>
       </c>
       <c r="N106" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="O106" s="6" t="inlineStr"/>
+      <c r="O106" s="6" t="inlineStr">
+        <is>
+          <t>Cơ sở 1: Báo giá nộp kèm</t>
+        </is>
+      </c>
       <c r="P106" s="6" t="inlineStr">
         <is>
           <t>Chưa mua sắm | Mua sắm để gia công bulong tháo nửa dưới hộp chèn hơi số 2 theo Văn bản khuyến cáo số 3360/EPS-PXSCC-VT | Vật tư đặt tên theo nguyên tắc chuẩn hóa, không tồn khoVật tư không có trong KHSXKD năm 2026</t>

</xml_diff>